<commit_message>
:sparkles: update doc tcc 1 and add referencias
</commit_message>
<xml_diff>
--- a/documentos - tcc/planilha-controle-de-leitura_excel.xlsx
+++ b/documentos - tcc/planilha-controle-de-leitura_excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iasmi\OneDrive\Documents\UFES\2024-2\TCC I\dados - datasus [repositorio git]\srag_tcc\documentos - tcc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B6C02A4-E562-48D0-88A8-DD3807DBA237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06F4733A-AC36-4D8B-9C9A-6C002AA7FA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1848" yWindow="1848" windowWidth="17280" windowHeight="8928" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -140,7 +140,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="47">
   <si>
     <t>Relevância com relação a temática</t>
   </si>
@@ -286,6 +286,18 @@
 entre os algoritmos Logistic Regression,
 Decision Tree e Random Forest</t>
   </si>
+  <si>
+    <t>https://repositorio.utfpr.edu.br/jspui/handle/1/26211</t>
+  </si>
+  <si>
+    <t>USO DE MACHINE LEARNING PARA PREVISÃO DA EVOLUÇÃO DE CASOS DE SRAG INCLUINDO CASOS DE COVID-19 CONSIDERANDO VARIÁVEIS CLÍNICAS E DEMOGRÁFICAS</t>
+  </si>
+  <si>
+    <t>AMAURI ORNELLAS DA SILVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Covid. Coronavirus. Machine learning. Classificação</t>
+  </si>
 </sst>
 </file>
 
@@ -397,7 +409,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -498,27 +510,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -589,6 +586,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -598,10 +598,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -932,7 +932,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="14.4">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
@@ -961,7 +961,7 @@
       <c r="W1" s="3"/>
     </row>
     <row r="2" spans="1:23" ht="14.4">
-      <c r="A2" s="25"/>
+      <c r="A2" s="26"/>
       <c r="B2" s="4"/>
       <c r="C2" s="2" t="s">
         <v>2</v>
@@ -988,7 +988,7 @@
       <c r="W2" s="3"/>
     </row>
     <row r="3" spans="1:23" ht="14.4">
-      <c r="A3" s="26"/>
+      <c r="A3" s="27"/>
       <c r="B3" s="5"/>
       <c r="C3" s="2" t="s">
         <v>3</v>
@@ -1272,7 +1272,7 @@
       <c r="W10" s="3"/>
     </row>
     <row r="11" spans="1:23" ht="100.8">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="24" t="s">
         <v>42</v>
       </c>
       <c r="B11" s="14" t="s">
@@ -1308,13 +1308,25 @@
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
     </row>
-    <row r="12" spans="1:23" ht="14.4">
-      <c r="A12" s="28"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
+    <row r="12" spans="1:23" ht="57.6">
+      <c r="A12" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="29">
+        <v>44428</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>43</v>
+      </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
@@ -25947,9 +25959,10 @@
     <hyperlink ref="F10" r:id="rId7" location="preview-link0 " xr:uid="{F6970C39-ABDF-42D5-9FEF-5E64FB0880A4}"/>
     <hyperlink ref="A11" r:id="rId8" display="https://www.scielosp.org/article/sdeb/2022.v46nspe8/118-129/pt/" xr:uid="{28181F7E-1D9B-45AC-ACA0-9D1E8E5F5461}"/>
     <hyperlink ref="F11" r:id="rId9" xr:uid="{52DDC651-910C-4DEA-9B2E-52D762DEDB2F}"/>
+    <hyperlink ref="F12" r:id="rId10" xr:uid="{04940FD5-431B-4602-B428-42F8EF9BF30E}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId10"/>
-  <legacyDrawing r:id="rId11"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
+  <legacyDrawing r:id="rId12"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
:memo: update tcc document
</commit_message>
<xml_diff>
--- a/documentos - tcc/planilha-controle-de-leitura_excel.xlsx
+++ b/documentos - tcc/planilha-controle-de-leitura_excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iasmi\OneDrive\Documents\UFES\2024-2\TCC I\dados - datasus [repositorio git]\srag_tcc\documentos - tcc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6229C35-0351-4AD8-B877-06A9ABB529FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D90AB2F0-BC67-4601-A8C4-159DBDF01606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-36" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -658,15 +658,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -681,6 +672,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -997,19 +997,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X996"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="41.33203125" style="16" customWidth="1"/>
-    <col min="3" max="3" width="17.33203125" customWidth="1"/>
-    <col min="4" max="4" width="33.88671875" style="16" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" customWidth="1"/>
-    <col min="6" max="6" width="17" style="16" customWidth="1"/>
-    <col min="7" max="7" width="85.88671875" style="16" customWidth="1"/>
-    <col min="8" max="24" width="8.6640625" customWidth="1"/>
+    <col min="2" max="2" width="41.28515625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" style="16" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" customWidth="1"/>
+    <col min="6" max="6" width="37.140625" style="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="85.85546875" style="16" customWidth="1"/>
+    <col min="8" max="24" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="14.4">
-      <c r="B1" s="30" t="s">
+    <row r="1" spans="1:24">
+      <c r="B1" s="36" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
@@ -1037,8 +1037,8 @@
       <c r="W1" s="3"/>
       <c r="X1" s="3"/>
     </row>
-    <row r="2" spans="1:24" ht="14.4">
-      <c r="B2" s="31"/>
+    <row r="2" spans="1:24">
+      <c r="B2" s="37"/>
       <c r="C2" s="4"/>
       <c r="D2" s="2" t="s">
         <v>2</v>
@@ -1064,8 +1064,8 @@
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
     </row>
-    <row r="3" spans="1:24" ht="14.4">
-      <c r="B3" s="32"/>
+    <row r="3" spans="1:24">
+      <c r="B3" s="38"/>
       <c r="C3" s="5"/>
       <c r="D3" s="2" t="s">
         <v>3</v>
@@ -1171,7 +1171,7 @@
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
     </row>
-    <row r="6" spans="1:24" ht="66">
+    <row r="6" spans="1:24" ht="51">
       <c r="A6" s="29">
         <v>2</v>
       </c>
@@ -1211,7 +1211,7 @@
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
     </row>
-    <row r="7" spans="1:24" ht="118.8">
+    <row r="7" spans="1:24" ht="114.75">
       <c r="A7" s="29">
         <v>3</v>
       </c>
@@ -1289,7 +1289,7 @@
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
     </row>
-    <row r="9" spans="1:24" ht="119.4">
+    <row r="9" spans="1:24" ht="115.5">
       <c r="A9" s="29">
         <v>5</v>
       </c>
@@ -1329,7 +1329,7 @@
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
     </row>
-    <row r="10" spans="1:24" ht="93">
+    <row r="10" spans="1:24" ht="90">
       <c r="A10" s="29">
         <v>6</v>
       </c>
@@ -1369,7 +1369,7 @@
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
     </row>
-    <row r="11" spans="1:24" ht="100.8">
+    <row r="11" spans="1:24" ht="105">
       <c r="A11" s="29">
         <v>7</v>
       </c>
@@ -1409,7 +1409,7 @@
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
     </row>
-    <row r="12" spans="1:24" ht="57.6">
+    <row r="12" spans="1:24" ht="75">
       <c r="A12" s="29">
         <v>8</v>
       </c>
@@ -1449,26 +1449,26 @@
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
     </row>
-    <row r="13" spans="1:24" ht="43.2">
-      <c r="A13" s="37">
+    <row r="13" spans="1:24" ht="45">
+      <c r="A13" s="34">
         <v>9</v>
       </c>
       <c r="B13" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="36" t="s">
+      <c r="C13" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="34" t="s">
+      <c r="D13" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="E13" s="35">
+      <c r="E13" s="32">
         <v>45392</v>
       </c>
-      <c r="F13" s="36" t="s">
+      <c r="F13" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="G13" s="33" t="s">
+      <c r="G13" s="30" t="s">
         <v>49</v>
       </c>
       <c r="H13" s="3"/>
@@ -1489,26 +1489,26 @@
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
     </row>
-    <row r="14" spans="1:24" ht="52.8">
-      <c r="A14" s="38">
+    <row r="14" spans="1:24" ht="51">
+      <c r="A14" s="35">
         <v>10</v>
       </c>
-      <c r="B14" s="36" t="s">
+      <c r="B14" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="36" t="s">
+      <c r="C14" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="36" t="s">
+      <c r="D14" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="E14" s="35">
+      <c r="E14" s="32">
         <v>43777</v>
       </c>
-      <c r="F14" s="36" t="s">
+      <c r="F14" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="G14" s="33" t="s">
+      <c r="G14" s="30" t="s">
         <v>48</v>
       </c>
       <c r="H14" s="3"/>
@@ -1529,7 +1529,7 @@
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
     </row>
-    <row r="15" spans="1:24" ht="14.4">
+    <row r="15" spans="1:24">
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -1554,7 +1554,7 @@
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
     </row>
-    <row r="16" spans="1:24" ht="14.4">
+    <row r="16" spans="1:24">
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>

</xml_diff>